<commit_message>
feat: publish full collection with 16 products
</commit_message>
<xml_diff>
--- a/thetaleofher_content_template.xlsx
+++ b/thetaleofher_content_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\The Tale Of Her\OneDrive\Documents\TTOH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTProject\Documents\Git\thetaleofher\Update\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EDB1FF-702A-404F-820E-EC817A6BCA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5003C62D-4CCF-4A1F-B11E-24C571B3D527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="19416" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="236">
   <si>
     <t>Field Key (Jangan Diubah)</t>
   </si>
@@ -592,6 +592,147 @@
   </si>
   <si>
     <t xml:space="preserve">Size S-M : Bust 95cm, length 63 cm. Size L-XL : Bust 120cm, length 70 cm.                                            Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.     </t>
+  </si>
+  <si>
+    <t>vittoria</t>
+  </si>
+  <si>
+    <t>Vittoria Shirt</t>
+  </si>
+  <si>
+    <t>White (#F2ECE1), Black (#241A1F)</t>
+  </si>
+  <si>
+    <t>Length 68 cm, bust 148 cm, shoulder 44 cm, arm 38 cm, sleeve 44 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>Elegant 3/4 sleeves and a statement collar bring a refined touch to this timeless silhouette. Designed with a relaxed fit for all-day comfort, it effortlessly combines sophistication with everyday ease.</t>
+  </si>
+  <si>
+    <t>assets/vittoria-white-1.jpg</t>
+  </si>
+  <si>
+    <t>assets/vittoria-white-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/vittoria-white-1.jpg, assets/vittoria-white-2.jpg, assets/vittoria-white-3.jpg, assets/vittoria-white-4.jpg, assets/vittoria-white-5.jpg, assets/vittoria-white-6.jpg, assets/vittoria-black-1.jpg, assets/vittoria-black-2.jpg, assets/vittoria-black-3.jpg, assets/vittoria-black-4.jpg, assets/vittoria-black-5.jpg, assets/vittoria-black-6.jpg</t>
+  </si>
+  <si>
+    <t>selena</t>
+  </si>
+  <si>
+    <t>Selena Shirt</t>
+  </si>
+  <si>
+    <t>Bust 126 cm, length 60 cm, shoulder 44 cm, arm 48 cm, sleeve 60 cm, waist 128 cm, hips 136 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>assets/selena-white-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/selena-white-1.jpg, assets/selena-white-2.jpg, assets/selena-white-3.jpg, assets/selena-white-4.jpg, assets/selena-white-5.jpg, assets/selena-white-6.jpg, assets/selena-black-1.jpg, assets/selena-black-2.jpg, assets/selena-black-3.jpg, assets/selena-black-4.jpg, assets/selena-black-5.jpg</t>
+  </si>
+  <si>
+    <t>sabria</t>
+  </si>
+  <si>
+    <t>Sabria Shirt</t>
+  </si>
+  <si>
+    <t>White (#F2ECE1)</t>
+  </si>
+  <si>
+    <t>Bust 120 cm, length 70 cm, shoulder 44 cm, arm 44 cm, sleeve 62 cm, waist 120 cm, hips 120 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>assets/sabria-white-1.jpg</t>
+  </si>
+  <si>
+    <t>assets/sabria-white-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/sabria-white-1.jpg, assets/sabria-white-2.jpg, assets/sabria-white-3.jpg, assets/sabria-white-4.jpg, assets/sabria-white-5.jpg, assets/sabria-white-6.jpg</t>
+  </si>
+  <si>
+    <t>erina</t>
+  </si>
+  <si>
+    <t>Erina Shirt</t>
+  </si>
+  <si>
+    <t>Bust 140 cm, length 75 cm, shoulder 44 cm, arm 50 cm, sleeve 65 cm, waist 144 cm, hips 150 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>assets/erina-white-1.jpg</t>
+  </si>
+  <si>
+    <t>assets/erina-white-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/erina-white-1.jpg, assets/erina-white-2.jpg, assets/erina-white-3.jpg, assets/erina-white-4.jpg, assets/erina-white-5.jpg, assets/erina-white-6.jpg</t>
+  </si>
+  <si>
+    <t>aurellia</t>
+  </si>
+  <si>
+    <t>Aurellia Shirt</t>
+  </si>
+  <si>
+    <t>Bust 124 cm, length 75 cm, shoulder 44 cm, arm 50 cm, sleeve 63 cm, waist 126 cm, hips 132 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>assets/aurellia-white-1.jpg</t>
+  </si>
+  <si>
+    <t>assets/aurellia-white-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/aurellia-white-1.jpg, assets/aurellia-white-2.jpg, assets/aurellia-white-3.jpg, assets/aurellia-white-4.jpg, assets/aurellia-white-5.jpg, assets/aurellia-white-6.jpg, assets/aurellia-black-1.jpg, assets/aurellia-black-2.jpg, assets/aurellia-black-3.jpg, assets/aurellia-black-4.jpg, assets/aurellia-black-5.jpg, assets/aurellia-black-6.jpg, assets/aurellia-black-7.jpg</t>
+  </si>
+  <si>
+    <t>camalia</t>
+  </si>
+  <si>
+    <t>Camalia Satin Blouse</t>
+  </si>
+  <si>
+    <t>blouses</t>
+  </si>
+  <si>
+    <t>Taupe (#B49C8A)</t>
+  </si>
+  <si>
+    <t>Bust 120 cm, length 72 cm, shoulder 46 cm, arm 58 cm, sleeve 65 cm, waist 126 cm, hips 132 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>assets/camalia-taupe-1.jpg</t>
+  </si>
+  <si>
+    <t>assets/camalia-taupe-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/camalia-taupe-1.jpg, assets/camalia-taupe-2.jpg, assets/camalia-taupe-3.jpg, assets/camalia-taupe-4.jpg, assets/camalia-taupe-5.jpg, assets/camalia-taupe-6.jpg</t>
+  </si>
+  <si>
+    <t>vienna</t>
+  </si>
+  <si>
+    <t>Vienna Shirt</t>
+  </si>
+  <si>
+    <t>White (#F2ECE1), Navy (#2B2F3A)</t>
+  </si>
+  <si>
+    <t>Bust 120 cm, length 65 cm, shoulder 50 cm, arm 56 cm, sleeve 30 cm, waist 120 cm, hips 120 cm. Measurements may vary by approx 1–2 cm. Unlined, non-sheer, no stretch.</t>
+  </si>
+  <si>
+    <t>assets/vienna-white-1.jpg</t>
+  </si>
+  <si>
+    <t>assets/vienna-white-2.jpg</t>
+  </si>
+  <si>
+    <t>assets/vienna-white-1.jpg, assets/vienna-white-2.jpg, assets/vienna-white-3.jpg, assets/vienna-white-4.jpg, assets/vienna-white-5.jpg, assets/vienna-white-6.jpg, assets/vienna-navy-1.jpg, assets/vienna-navy-2.jpg, assets/vienna-navy-3.jpg, assets/vienna-navy-4.jpg, assets/vienna-navy-5.jpg, assets/vienna-navy-6.jpg</t>
   </si>
 </sst>
 </file>
@@ -611,11 +752,13 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -996,14 +1139,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1017,7 +1160,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1031,7 +1174,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -1045,7 +1188,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -1059,7 +1202,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
@@ -1073,7 +1216,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1087,7 +1230,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -1101,7 +1244,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
@@ -1115,7 +1258,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
@@ -1129,7 +1272,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>36</v>
       </c>
@@ -1143,7 +1286,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>40</v>
       </c>
@@ -1157,7 +1300,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="32" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
@@ -1179,7 +1322,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -1188,7 +1331,7 @@
     <col min="6" max="6" width="31" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
@@ -1208,7 +1351,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="48" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
@@ -1228,7 +1371,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="48" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>60</v>
       </c>
@@ -1244,7 +1387,7 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" ht="48" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>64</v>
       </c>
@@ -1264,7 +1407,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>70</v>
       </c>
@@ -1287,22 +1430,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:O18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="36" customWidth="1"/>
     <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="40.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="40.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="11" width="60" customWidth="1"/>
     <col min="12" max="13" width="31" customWidth="1"/>
     <col min="14" max="14" width="60" customWidth="1"/>
     <col min="15" max="15" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>74</v>
       </c>
@@ -1349,24 +1492,24 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="64" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" ht="75" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>189</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D2" s="2">
-        <v>366000</v>
+        <v>329000</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>121</v>
+        <v>191</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>91</v>
@@ -1375,45 +1518,45 @@
         <v>92</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>178</v>
+        <v>192</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>193</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>93</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>122</v>
+        <v>194</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>123</v>
+        <v>195</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>124</v>
+        <v>196</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="64" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>125</v>
+        <v>197</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>89</v>
       </c>
       <c r="D3" s="3">
-        <v>365000</v>
+        <v>329000</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>90</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>127</v>
+        <v>191</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>91</v>
@@ -1422,7 +1565,7 @@
         <v>92</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>182</v>
+        <v>199</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>95</v>
@@ -1431,45 +1574,43 @@
         <v>93</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>128</v>
+        <v>59</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>129</v>
+        <v>200</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>130</v>
+        <v>201</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="64" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" ht="75" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>131</v>
+        <v>202</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>132</v>
+        <v>203</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="D4" s="2">
-        <v>450000</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>99</v>
-      </c>
+        <v>369000</v>
+      </c>
+      <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>174</v>
+        <v>91</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>172</v>
+        <v>92</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>183</v>
+        <v>205</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>96</v>
@@ -1478,45 +1619,43 @@
         <v>93</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>136</v>
+        <v>206</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>138</v>
+        <v>208</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="64" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" ht="60" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>139</v>
+        <v>209</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>141</v>
+        <v>89</v>
       </c>
       <c r="D5" s="3">
-        <v>345000</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>90</v>
-      </c>
+        <v>339000</v>
+      </c>
+      <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>175</v>
+        <v>204</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>91</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>173</v>
+        <v>92</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>97</v>
@@ -1525,45 +1664,45 @@
         <v>93</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>142</v>
+        <v>212</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>143</v>
+        <v>213</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>144</v>
+        <v>214</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="64" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" ht="90" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>145</v>
+        <v>215</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>146</v>
+        <v>216</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>141</v>
+        <v>89</v>
       </c>
       <c r="D6" s="2">
-        <v>348000</v>
+        <v>369000</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>90</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>173</v>
+        <v>91</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>188</v>
+        <v>217</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>98</v>
@@ -1572,36 +1711,36 @@
         <v>93</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>147</v>
+        <v>218</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>148</v>
+        <v>219</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>149</v>
+        <v>220</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="48" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" ht="60" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>150</v>
+        <v>221</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>151</v>
+        <v>222</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>89</v>
+        <v>223</v>
       </c>
       <c r="D7" s="3">
-        <v>352000</v>
+        <v>355000</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>177</v>
+        <v>224</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>91</v>
@@ -1610,7 +1749,7 @@
         <v>100</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>184</v>
+        <v>225</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>101</v>
@@ -1619,45 +1758,43 @@
         <v>93</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>152</v>
+        <v>226</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>153</v>
+        <v>227</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>154</v>
+        <v>228</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="48" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" ht="75" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>229</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>156</v>
+        <v>230</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D8" s="2">
-        <v>315000</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>90</v>
-      </c>
+        <v>319000</v>
+      </c>
+      <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>176</v>
+        <v>231</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>100</v>
+      <c r="H8" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>185</v>
+        <v>232</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>102</v>
@@ -1666,122 +1803,448 @@
         <v>93</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>157</v>
+        <v>233</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>158</v>
+        <v>234</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>159</v>
+        <v>235</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="48" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="D9" s="4">
-        <v>442000</v>
-      </c>
-      <c r="E9" s="4" t="s">
+    <row r="9" spans="1:15" ht="60" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="2">
+        <v>366000</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="G9" s="4" t="s">
+      <c r="F9" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>179</v>
+      <c r="H9" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>102</v>
+        <v>181</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>178</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>93</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>162</v>
+        <v>122</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>163</v>
+        <v>123</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="O9" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="48" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:15" ht="60" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="3">
+        <v>365000</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D11" s="2">
+        <v>450000</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="60" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" s="3">
+        <v>345000</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="60" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="2">
+        <v>348000</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="60" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="3">
+        <v>352000</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="45" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="2">
+        <v>315000</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="45" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D16" s="4">
+        <v>442000</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="45" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B17" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D17" s="5">
         <v>475000</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F17" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G17" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H17" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I17" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K17" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L17" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M17" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N17" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O17" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.35">
-      <c r="J14" s="2"/>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1791,7 +2254,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -1799,7 +2262,7 @@
     <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>103</v>
       </c>
@@ -1813,7 +2276,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="96" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="105" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1827,7 +2290,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="160" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="165" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1841,7 +2304,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="112" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="105" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1855,7 +2318,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="80" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="75" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>

</xml_diff>